<commit_message>
change excel column name, add toast when count finish, increase download button size
</commit_message>
<xml_diff>
--- a/src/app/api/[reportId]/Asset_Report_edit.xlsx
+++ b/src/app/api/[reportId]/Asset_Report_edit.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c6058d78e55bea86/เอกสาร/Asset count/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A19780D7-57E2-4836-B572-ED6AA77D445D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{A19780D7-57E2-4836-B572-ED6AA77D445D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71064549-BC5D-4C44-A010-324B7E010DE2}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="24792" windowHeight="14856" xr2:uid="{4495CCDA-79BA-4027-8A10-C93A0DF9419C}"/>
   </bookViews>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -86,9 +84,6 @@
     <t>Count Check</t>
   </si>
   <si>
-    <t>Assign Not Correct</t>
-  </si>
-  <si>
     <t>Asset Damaged</t>
   </si>
   <si>
@@ -105,6 +100,9 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>Assign Incorrect</t>
   </si>
 </sst>
 </file>
@@ -658,13 +656,13 @@
         <v>15</v>
       </c>
       <c r="F11" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G11" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="H11" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="24.9" customHeight="1" x14ac:dyDescent="0.4">
@@ -672,16 +670,16 @@
         <v>1</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>22</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>

</xml_diff>